<commit_message>
Sesión 6: A1 corregida (Cancillería con variantes + UNCTAD), A3 con ACE de la ALADI, correcciones de la revisión de G
- A1: filtro de canje de notas corregido; búsqueda con variantes de nombre y por tipo
  de acuerdo; cruce con UNCTAD país por país. Francia pasa a NO; Bélgica y Luxemburgo
  quedan en revisión completa por diferencia entre fuentes.
- A3: instrumento concreto por país (ACE de la ALADI). Panamá NO (ACE 76).
- C2 con dimensiones disponibles (CRI, HND, JAM, PAN, SUR, GTM) y Canadá A5 como alerta.
- Panamá A3, Guatemala C2 y Luxemburgo C4 aprobadas por G.
- Planillas solo con pendientes: quedan revision_bases_64_paises y revision_tanda2_america.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzD7QUUB49X53DnDPTty9t
</commit_message>
<xml_diff>
--- a/data/revision/revision_tanda2_america.xlsx
+++ b/data/revision/revision_tanda2_america.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resto" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Revisión completa'!$A$1:$O$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Muestreo'!$A$1:$O$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Resto'!$A$1:$O$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Revisión completa'!$A$1:$O$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Muestreo'!$A$1:$O$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Resto'!$A$1:$O$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -551,21 +551,21 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>- Revisión completa (12 filas): Revisar todas: respuestas interpretativas, en null, fuera del cálculo y todas las condiciones críticas (⚡).</t>
+          <t>- Revisión completa (1 filas): Revisar todas: respuestas interpretativas, en null, fuera del cálculo y todas las condiciones críticas (⚡).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>- Muestreo (4 filas): Para cada pregunta mecánica, 4 países al azar: abrí el link y verificá el dato.</t>
+          <t>- Muestreo (0 filas): Para cada pregunta mecánica, 4 países al azar: abrí el link y verificá el dato.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>- Resto (76 filas): Solo como referencia. Se pueden aprobar, pero no hace falta revisarlas una por una.</t>
+          <t>- Resto (58 filas): Solo como referencia. Se pueden aprobar, pero no hace falta revisarlas una por una.</t>
         </is>
       </c>
     </row>
@@ -582,56 +582,14 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>- Barbados A5: Cambio retroactivo documentado por la autoridad tributaria; alcanza a los grupos multinacionales, incluidos los extranjeros. Es la aplicación de un estándar de la OCDE que otros países también adoptaron con efecto retroactivo: REVISAR si se acepta.</t>
+          <t>- Canadá A5: Corrección pedida en la revisión de G (planilla revision_tanda2_america, 28/10/2026): como la ley retroactiva se derogó y se devolvió lo cobrado, no cuenta como cambio retroactivo vigente (NO) y se publica como alerta. Reemplaza, para estos casos, el criterio 17 de la sesión 5. A CONFIRMAR.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>- Canadá I3-2: Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado). Casos revisados y no contados: la incautación de un avión de carga ruso en 2023 (sanción internacional; criterio aprobado en la sesión 5) y la ley de Quebec de 2022 que revocó las licencias de exploración de hidrocarburos con un programa de indemnización de gastos. La ley de Quebec no es una expropiación formal; los fundadores pueden decidir si la revocación de licencias cuenta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>- Cuba A5: Se tomó como cambio retroactivo porque alcanza a fondos depositados antes de la medida. No hay norma publicada: la información viene de fuentes de EFE. REVISAR.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>- México A5: El Gobierno fundó la cancelación en la falta de inversión mínima (2017-2021); se tomó como cambio con efecto retroactivo por aplicarse a concesiones previas a la reforma. La reforma eléctrica de marzo de 2021 (revisión retroactiva de contratos) queda fuera de la ventana de 5 años. REVISAR.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>- México G4: Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras. En el tablero de la semana relevada solo figuran 2 partidas a México: REVISAR si la frecuencia se recupera después de las obras.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>- Panamá A5: Criterio aprobado: cuenta una decisión de un tribunal supremo con efecto retroactivo sobre empresas. Esta decisión alcanzó a una empresa extranjera en particular y no tiene efecto general: REVISAR.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
           <t>- Estados Unidos C3: Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Caso revisado y no contado: en noviembre de 2022 EE.UU. impuso derechos antidumping a los tubos OCTG argentinos que exporta Siderca (grupo Techint), y Argentina llevó el caso a la OMC (DS617). Criterio aprobado (sesión 5): las medidas antidumping no cuentan como discriminación, salvo que un fallo de la OMC las declare incompatibles. El panel entregó su informe a las partes el 02/05/2025, pero a pedido de ambas su publicación se postergó hasta el 29/10/2026: todavía no hay fallo público. REVISAR DESPUÉS DEL 29/10/2026: si el informe declara la medida incompatible, la respuesta pasa a SÍ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>- Estados Unidos A5: Se tomó como cambio regulatorio retroactivo la suspensión de un proyecto con permisos ya otorgados. Es una orden administrativa sobre un proyecto, no una norma general: REVISAR si se acepta.</t>
         </is>
       </c>
     </row>
@@ -647,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -753,12 +711,12 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Barbados</t>
+          <t>Canadá</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>BRB</t>
+          <t>CAN</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -773,37 +731,38 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>SÍ ⚡</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>La Ley del Impuesto Complementario a las Sociedades 2024 (Corporation Top-up Tax Act 2024-16), que aplica el impuesto mínimo global de 15% (Pilar Dos de la OCDE), rige en forma retroactiva para los ejercicios iniciados desde el 31/12/2023.</t>
+          <t>La Ley del Impuesto sobre los Servicios Digitales (sanción del 20/06/2024) creó un impuesto de 3% sobre ingresos digitales de grandes empresas, en su mayoría extranjeras, con efecto retroactivo al 01/01/2022. La Ley de Implementación del Presupuesto 2025 n.º 1 (S.C. 2026, c. 3, art. 126), sancionada el 26/03/2026, lo derogó con efecto al 20/06/2024 y ordenó devolver lo cobrado.</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>impuesto mínimo a grandes empresas sancionado en 2024 con efecto retroactivo al ejercicio 2024 (dato 2024, Barbados Revenue Authority)</t>
+          <t>impuesto retroactivo a los servicios digitales derogado en 2026, con devolución de lo cobrado (dato 2026, BLG)</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>https://www.bra.gov.bb/About/Legislation-Regulations/Corporation-Top-up-Tax-Act-2024-16</t>
+          <t>https://www.blg.com/en/insights/2024/07/canadas-unilateral-digital-services-tax-forges-ahead-with-retroactive-effect</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>Barbados Revenue Authority, Corporation Top-up Tax Act 2024-16 · 2026-10-28</t>
+          <t>BLG (Borden Ladner Gervais), "Canada’s unilateral Digital Services Tax forges ahead with retroactive effect" (10/07/2024) · 2026-10-28</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>Cambio retroactivo documentado por la autoridad tributaria; alcanza a los grupos multinacionales, incluidos los extranjeros. Es la aplicación de un estándar de la OCDE que otros países también adoptaron con efecto retroactivo: REVISAR si se acepta.</t>
+          <t>Corrección pedida en la revisión de G (planilla revision_tanda2_america, 28/10/2026): como la ley retroactiva se derogó y se devolvió lo cobrado, no cuenta como cambio retroactivo vigente (NO) y se publica como alerta. Reemplaza, para estos casos, el criterio 17 de la sesión 5. A CONFIRMAR.</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>Búsqueda web ("Bahamas OR Barbados OR St Lucia OR Antigua … retroactive tax OR legislation foreign companies 2022-2026") (https://www.businessbarbados.com/articles/barbados-still-open-for-business-in-a-maturing-tax-environment): Solo Barbados tiene un cambio retroactivo documentado.</t>
+          <t>Gobierno de Canadá, Justice Laws, Budget 2025 Implementation Act, No. 1 (S.C. 2026, c. 3), art. 126 (https://laws-lois.justice.gc.ca/eng/acts/B-9.8598/FullText.html): Deroga la Ley del Impuesto sobre los Servicios Digitales con efecto al 20/06/2024; sancionada el 26/03/2026.
+PwC Canadá, "Canada intends to rescind its Digital Services Tax Act" (2025) (https://www.pwc.com/ca/en/services/tax/publications/tax-insights/canada-digital-services-tax-act-2025.html): Confirma el efecto retroactivo y el anuncio de derogación de junio de 2025.</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr">
@@ -816,813 +775,23 @@
       <c r="O2" s="6" t="n"/>
       <c r="P2" s="4" t="inlineStr">
         <is>
-          <t>8268fba1d0fc</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Canadá</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>CAN</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>A5</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo cambios regulatorios retroactivos documentados en los últimos 5 años, en cualquier sector, que afectaran a empresas extranjeras?</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>SÍ ⚡</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>La Ley del Impuesto sobre los Servicios Digitales (sanción del 20/06/2024) creó un impuesto de 3% sobre ingresos digitales de grandes empresas, en su mayoría extranjeras, con efecto retroactivo al 01/01/2022. La Ley de Implementación del Presupuesto 2025 n.º 1 (S.C. 2026, c. 3, art. 126), sancionada el 26/03/2026, lo derogó con efecto al 20/06/2024 y ordenó devolver lo cobrado.</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>impuesto a los servicios digitales sancionado en 2024 con efecto retroactivo a 2022, luego derogado en 2026 (dato 2024, BLG)</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>https://www.blg.com/en/insights/2024/07/canadas-unilateral-digital-services-tax-forges-ahead-with-retroactive-effect</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>BLG (Borden Ladner Gervais), "Canada’s unilateral Digital Services Tax forges ahead with retroactive effect" (10/07/2024) · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Criterio aprobado (sesión 5): una ley retroactiva que después se derogó sigue contando, porque existió; el dato publicado aclara la derogación. La derogación se declaró vigente desde el 20/06/2024, el mismo día de la sanción, y se ordenó devolver lo pagado.</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>Gobierno de Canadá, Justice Laws, Budget 2025 Implementation Act, No. 1 (S.C. 2026, c. 3), art. 126 (https://laws-lois.justice.gc.ca/eng/acts/B-9.8598/FullText.html): Deroga la Ley del Impuesto sobre los Servicios Digitales con efecto al 20/06/2024; sancionada el 26/03/2026.
-PwC Canadá, "Canada intends to rescind its Digital Services Tax Act" (2025) (https://www.pwc.com/ca/en/services/tax/publications/tax-insights/canada-digital-services-tax-act-2025.html): Confirma el efecto retroactivo y el anuncio de derogación de junio de 2025.</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M3" s="6" t="n"/>
-      <c r="N3" s="6" t="n"/>
-      <c r="O3" s="6" t="n"/>
-      <c r="P3" s="4" t="inlineStr">
-        <is>
-          <t>9a5782500501</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Cuba</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>CUB</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>A5</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo cambios regulatorios retroactivos documentados en los últimos 5 años, en cualquier sector, que afectaran a empresas extranjeras?</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>SÍ ⚡</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>En noviembre de 2025 el Gobierno dejó de permitir que las empresas extranjeras retiren o transfieran al exterior las divisas que ya tenían depositadas en bancos cubanos ("corralito"), según fuentes de EFE.</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>bloqueo de las divisas ya depositadas por empresas extranjeras (dato 2025, Emol (EFE))</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>https://www.emol.com/noticias/Economia/2025/11/21/1183911/corralito-cuba-empresas-extranjeras.html</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>Emol (EFE), "Corralito en Cuba: Gobierno está impidiendo a empresas extranjeras el retiro y envío de divisas al exterior" (21/11/2025) · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Se tomó como cambio retroactivo porque alcanza a fondos depositados antes de la medida. No hay norma publicada: la información viene de fuentes de EFE. REVISAR.</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>Diario El Mundo (El Salvador), Cuba congela divisas de empresas extranjeras (https://diario.elmundo.sv/economia/cuba-congela-divisas-de-empresas-extranjeras-y-extiende-restricciones-bancarias-en-medio-de-crisis-economica): Confirma la medida.</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M4" s="6" t="n"/>
-      <c r="N4" s="6" t="n"/>
-      <c r="O4" s="6" t="n"/>
-      <c r="P4" s="4" t="inlineStr">
-        <is>
-          <t>2bbfe415546d</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Estados Unidos</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>A5</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo cambios regulatorios retroactivos documentados en los últimos 5 años, en cualquier sector, que afectaran a empresas extranjeras?</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>SÍ ⚡</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>El 22/08/2025 la Oficina de Gestión de Energía Oceánica (BOEM) ordenó detener la construcción del parque eólico marino Revolution Wind, de la danesa Ørsted, que tenía todos los permisos federales y estatales aprobados y estaba 80% construido.</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>orden de frenar un parque eólico marino de una empresa extranjera que ya tenía sus permisos aprobados (dato 2025, Ørsted)</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>https://orsted.com/en/company-announcement-list/2025/08/revolution-wind-receives-offshore-stop-work-order--145387701</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>Ørsted, anuncio a la bolsa "Revolution Wind receives offshore stop-work order" (22/08/2025) · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>Se tomó como cambio regulatorio retroactivo la suspensión de un proyecto con permisos ya otorgados. Es una orden administrativa sobre un proyecto, no una norma general: REVISAR si se acepta.</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>UConn Digital Journalism, cronología de la orden de Revolution Wind (https://digitaljournalism.uconn.edu/balance-of-power/2026/01/08/revolution-wind-stop-work-order/): La orden invoca la revisión dispuesta por el memorando presidencial del 20/01/2025.</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M5" s="6" t="n"/>
-      <c r="N5" s="6" t="n"/>
-      <c r="O5" s="6" t="n"/>
-      <c r="P5" s="4" t="inlineStr">
-        <is>
-          <t>ef5503db479c</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Honduras</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>HND</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>A5</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo cambios regulatorios retroactivos documentados en los últimos 5 años, en cualquier sector, que afectaran a empresas extranjeras?</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>SÍ ⚡</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>En abril de 2022 el Congreso derogó la ley de Zonas de Empleo y Desarrollo Económico (ZEDE) y quitó su base constitucional (Decretos 32-2022 y 33-2022), con aplicación inmediata. Los inversores de la ZEDE Próspera (EE.UU.) tenían acuerdos de estabilidad jurídica firmados en 2021 y reclaman ante el CIADI.</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>derogación de las zonas económicas especiales que afectó acuerdos de estabilidad de inversores extranjeros (dato 2022, IISD)</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>https://www.iisd.org/itn/es/2026/09/09/tribunal-del-ciadi-rechaza-intento-de-honduras-de-condicionar-su-consentimiento-a-arbitraje-en-el-cafta-dr-al-agotamiento-de-los-recursos-internos-ifeoluwa-oyemade/</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>IISD, Investment Treaty News, decisión del CIADI en el caso Próspera contra Honduras (09/09/2026) · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>Cambio con efecto sobre acuerdos de estabilidad ya firmados por inversores extranjeros.</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>Revista E&amp;N, reclamo de Próspera contra Honduras (https://www.revistaeyn.com/empresasymanagement/prosperazede-redujo-85-el-monto-reclamado-en-arbitraje-contra-honduras-IK27873597): El monto reclamado bajó de US$10.775 millones a US$1.630 millones.</t>
-        </is>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M6" s="6" t="n"/>
-      <c r="N6" s="6" t="n"/>
-      <c r="O6" s="6" t="n"/>
-      <c r="P6" s="4" t="inlineStr">
-        <is>
-          <t>0f5dc886c705</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>MEX</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>A5</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo cambios regulatorios retroactivos documentados en los últimos 5 años, en cualquier sector, que afectaran a empresas extranjeras?</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>SÍ ⚡</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>La reforma a la Ley Minera de abril de 2022 declaró el litio patrimonio de la nación y reservó su explotación al Estado. En 2023 el Gobierno canceló nueve concesiones de Ganfeng y sus filiales británicas Bacanora Lithium y Sonora Lithium, otorgadas antes del cambio; la cámara minera Camimex sostuvo que la ley no es retroactiva y que los permisos eran anteriores.</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>cancelación de concesiones de litio de empresas extranjeras otorgadas antes de la reforma de 2022 (dato 2023, Bloomberg Línea)</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>https://www.bloomberglinea.com/latinoamerica/mexico/minera-china-ganfeng-demanda-a-mexico-por-cancelar-concesiones-de-litio/</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>Bloomberg Línea, "Minera china Ganfeng demanda a México por cancelar concesiones de litio" (25/06/2024) · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>El Gobierno fundó la cancelación en la falta de inversión mínima (2017-2021); se tomó como cambio con efecto retroactivo por aplicarse a concesiones previas a la reforma. La reforma eléctrica de marzo de 2021 (revisión retroactiva de contratos) queda fuera de la ventana de 5 años. REVISAR.</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>Forbes Colombia, reforma eléctrica de México (03/03/2021) (https://forbes.co/2021/03/03/actualidad/no-queremos-expropiar-por-expropiar-afirma-amlo-tras-reforma-electrica/): Ordenó revisar en forma retroactiva contratos con productores privados, pero es de marzo de 2021, fuera de la ventana.
-Xataka México, cancelación de concesiones de litio (https://www.xataka.com.mx/automovil/mexico-cancela-masivas-concesiones-litio-para-baterias-autos-electricos-china-ha-dado-paso-obvio-demandar): Confirma la cancelación de las concesiones de Ganfeng.</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M7" s="6" t="n"/>
-      <c r="N7" s="6" t="n"/>
-      <c r="O7" s="6" t="n"/>
-      <c r="P7" s="4" t="inlineStr">
-        <is>
-          <t>2f65cdf19917</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Panamá</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>PAN</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>A5</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo cambios regulatorios retroactivos documentados en los últimos 5 años, en cualquier sector, que afectaran a empresas extranjeras?</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>SÍ ⚡</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>El 28/11/2023 la Corte Suprema de Justicia declaró inconstitucional la Ley 406 de 2023, que aprobaba el contrato de concesión de Minera Panamá (filial de la canadiense First Quantum); el Gobierno anunció el cierre de la mina.</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>la Corte Suprema anuló la ley del contrato de una minera extranjera y la mina cerró (dato 2023, Voz de América)</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>https://www.vozdeamerica.com/a/corte-suprema-de-justicia-de-panama-declara-inconstitucional-polemico-contrato-minero/7373295.html</t>
-        </is>
-      </c>
-      <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t>Voz de América, "Corte Suprema de Justicia de Panamá declara inconstitucional polémico contrato minero" (28/11/2023) · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J8" s="4" t="inlineStr">
-        <is>
-          <t>Criterio aprobado: cuenta una decisión de un tribunal supremo con efecto retroactivo sobre empresas. Esta decisión alcanzó a una empresa extranjera en particular y no tiene efecto general: REVISAR.</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>La República, fallo sobre el contrato de First Quantum (https://www.larepublica.co/globoeconomia/la-corte-suprema-de-panama-declara-inconstitucional-contrato-minero-con-canadiense-first-quantum-3757247): Confirma la declaración de inconstitucionalidad de toda la Ley 406.</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M8" s="6" t="n"/>
-      <c r="N8" s="6" t="n"/>
-      <c r="O8" s="6" t="n"/>
-      <c r="P8" s="4" t="inlineStr">
-        <is>
-          <t>db7dc47b124d</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>MEX</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>G4</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>En septiembre de 2026 salieron 38 vuelos regulares con pasajeros desde aeropuertos argentinos a México (8,9 por semana en promedio; AEROVIAS DE MEXICO - AEROMEXICO, AEROLINEAS ARGENTINAS SA).</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>9 vuelos directos por semana en promedio desde Argentina (dato 2026, ANAC)</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras. En el tablero de la semana relevada solo figuran 2 partidas a México: REVISAR si la frecuencia se recupera después de las obras.</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 38 despegues regulares con pasajeros a México en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 2 partidas a México entre el 26/10 y el 01/11/2026.</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M9" s="6" t="n"/>
-      <c r="N9" s="6" t="n"/>
-      <c r="O9" s="6" t="n"/>
-      <c r="P9" s="4" t="inlineStr">
-        <is>
-          <t>8967ff62fb7c</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Belice</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>BLZ</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>SÍ ⚡</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>El 27/08/2024 el Ministro de Recursos Naturales firmó, con aprobación del Gabinete, el aviso de expropiación (adquisición forzosa) de la extensión de 24 acres de la isla Stake Bank, en disputa judicial; el Tribunal Superior declaró constitucional la adquisición y el caso está en apelación.</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>expropiación de la extensión de la isla Stake Bank (dato 2024, Gobierno de Belice)</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>https://www.pressoffice.gov.bz/disputed-stakebank-extension-to-be-acquired-by-gob-for-a-public-purpose/</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>Gobierno de Belice, oficina de prensa, "Disputed Stakebank Extension to be Acquired by GOB for a Public Purpose" (27/08/2024) · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>Expropiación documentada por el propio Gobierno dentro de la ventana de 10 años.</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 0 casos con Belice como demandado (0 pendientes).
-Gobierno de Belice, comunicado del 12/03/2026 (https://www.pressoffice.gov.bz/wp-content/uploads/2026/03/Mar-12-PR071-26-Statement-by-the-Government-of-Belize.pdf): El Tribunal Superior declaró constitucional la adquisición; hay apelación.</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M10" s="6" t="n"/>
-      <c r="N10" s="6" t="n"/>
-      <c r="O10" s="6" t="n"/>
-      <c r="P10" s="4" t="inlineStr">
-        <is>
-          <t>2f041e8e7669</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Canadá</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>CAN</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 16 casos contra Canadá (4 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado). Casos revisados y no contados: la incautación de un avión de carga ruso en 2023 (sanción internacional; criterio aprobado en la sesión 5) y la ley de Quebec de 2022 que revocó las licencias de exploración de hidrocarburos con un programa de indemnización de gastos. La ley de Quebec no es una expropiación formal; los fundadores pueden decidir si la revocación de licencias cuenta.</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 16 casos con Canadá como demandado (4 pendientes).
-Gobierno de Canadá, Global Affairs, incautación de un avión de carga ruso en Toronto (junio de 2023) (https://www.canada.ca/en/global-affairs/news/2023/06/government-of-canada-orders-seizure-of-russian-registered-cargo-aircraft-at-toronto-pearson-airport.html): Incautación de un Antonov An-124 de Volga-Dnepr por sanciones. No cuenta (sanción internacional).
-Búsqueda web ("Canada expropriation OR nationalization of company assets 2017-2026") (https://canadians.org/analysis/abitibibowater-files-nafta-challenge/): La expropiación de AbitibiBowater es de 2008-2010, fuera de la ventana.
-Gobierno de Quebec, ley que pone fin a la investigación y producción de hidrocarburos (sancionada el 13/04/2022) (https://www.quebec.ca/nouvelles/actualites/details/transition-energetique-quebec-met-fin-a-la-recherche-et-a-la-production-dhydrocarbures-sur-son-territoire-39395): Revocó las licencias de exploración vigentes, con un programa de indemnización de gastos (Decreto 1314-2022).</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M11" s="6" t="n"/>
-      <c r="N11" s="6" t="n"/>
-      <c r="O11" s="6" t="n"/>
-      <c r="P11" s="4" t="inlineStr">
-        <is>
-          <t>55aee5a215be</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>MEX</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>SÍ ⚡</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>La reforma a la Ley Minera de abril de 2022 nacionalizó el litio: lo declaró patrimonio de la nación, reservó su explotación al Estado y creó la empresa estatal LitioMx. En 2023 el Gobierno canceló nueve concesiones de Ganfeng y sus filiales británicas.</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>nacionalización del litio y cancelación de concesiones de una minera extranjera (dato 2023, Bloomberg Línea)</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>https://www.bloomberglinea.com/latinoamerica/mexico/minera-china-ganfeng-demanda-a-mexico-por-cancelar-concesiones-de-litio/</t>
-        </is>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>Bloomberg Línea, "Minera china Ganfeng demanda a México por cancelar concesiones de litio" (25/06/2024) · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>Nacionalización sectorial documentada dentro de la ventana de 10 años. También se revisó la ocupación temporal de 120 km de vías de Ferrosur (Grupo México, mayo de 2023), que el Gobierno no calificó como expropiación.</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>El Financiero, "No estamos expropiando nada": ocupación de vías de Ferrosur (20/05/2023) (https://www.elfinanciero.com.mx/nacional/2023/05/20/no-estamos-expropiando-nada-adan-augusto-sobre-toma-de-ferrosur/): Decreto de ocupación temporal; el Gobierno negó que fuera expropiación.
-CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 58 casos con México como demandado (20 pendientes).</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M12" s="6" t="n"/>
-      <c r="N12" s="6" t="n"/>
-      <c r="O12" s="6" t="n"/>
-      <c r="P12" s="4" t="inlineStr">
-        <is>
-          <t>b876ecfe1913</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Nicaragua</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>NIC</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>SÍ ⚡</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>En marzo de 2023 el Gobierno disolvió el Consejo Superior de la Empresa Privada (COSEP) y confiscó su sede en Managua; según el Observatorio OPTA, a abril de 2024 había 35 cámaras empresariales cerradas y confiscaciones de inmuebles, empresas y medios.</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>confiscación de la sede de la principal cámara empresarial y de bienes de empresas y medios (dato 2023, Confidencial)</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>https://confidencial.digital/?p=100783</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>Confidencial, informe del Observatorio OPTA sobre confiscaciones en Nicaragua (mayo de 2024) · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>Confiscaciones documentadas dentro de la ventana de 10 años.</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 3 casos con Nicaragua como demandado (0 pendientes).
-La Tercera, confiscación de bienes de 222 expresos políticos desterrados (https://www.latercera.com/mundo/noticia/gobierno-de-nicaragua-confisca-bienes-a-222-expresos-politicos-desterrados-a-estados-unidos/2BVGSQEXB5G2NINO35WNIMRPHE/): Sentencia que ordenó confiscar todos los inmuebles de 222 opositores.</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M13" s="6" t="n"/>
-      <c r="N13" s="6" t="n"/>
-      <c r="O13" s="6" t="n"/>
-      <c r="P13" s="4" t="inlineStr">
-        <is>
-          <t>e23350dd4f0b</t>
+          <t>244cc2c1ef00</t>
         </is>
       </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
-  <autoFilter ref="A1:O13"/>
+  <autoFilter ref="A1:O2"/>
   <dataValidations count="2">
-    <dataValidation sqref="M2:M13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Aprobado" error="Elegí &quot;sí&quot; o &quot;no&quot;." type="list">
+    <dataValidation sqref="M2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Aprobado" error="Elegí &quot;sí&quot; o &quot;no&quot;." type="list">
       <formula1>"sí,no"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revisó" error="Elegí G (Giuliano) o A (Agustina)." type="list">
+    <dataValidation sqref="N2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revisó" error="Elegí G (Giuliano) o A (Agustina)." type="list">
       <formula1>"G,A"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1634,7 +803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1737,307 +906,17 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Belice</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>BLZ</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>G4</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a Belice. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
-        </is>
-      </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a Belice en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a Belice entre el 26/10 y el 01/11/2026.</t>
-        </is>
-      </c>
-      <c r="L2" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M2" s="6" t="n"/>
-      <c r="N2" s="6" t="n"/>
-      <c r="O2" s="6" t="n"/>
-      <c r="P2" s="4" t="inlineStr">
-        <is>
-          <t>4a8338505c61</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Canadá</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>CAN</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>G4</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a Canadá. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a Canadá en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a Canadá entre el 26/10 y el 01/11/2026.</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M3" s="6" t="n"/>
-      <c r="N3" s="6" t="n"/>
-      <c r="O3" s="6" t="n"/>
-      <c r="P3" s="4" t="inlineStr">
-        <is>
-          <t>8e1188be47bf</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Costa Rica</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>CRI</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>G4</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a Costa Rica. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a Costa Rica en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a Costa Rica entre el 26/10 y el 01/11/2026.</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M4" s="6" t="n"/>
-      <c r="N4" s="6" t="n"/>
-      <c r="O4" s="6" t="n"/>
-      <c r="P4" s="4" t="inlineStr">
-        <is>
-          <t>861b64c1e9d3</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>San Vicente y las Granadinas</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>VCT</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>G4</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a San Vicente y las Granadinas. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a San Vicente y las Granadinas en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a San Vicente y las Granadinas entre el 26/10 y el 01/11/2026.</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M5" s="6" t="n"/>
-      <c r="N5" s="6" t="n"/>
-      <c r="O5" s="6" t="n"/>
-      <c r="P5" s="4" t="inlineStr">
-        <is>
-          <t>13e991a02165</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
-  <autoFilter ref="A1:O5"/>
+  <autoFilter ref="A1:O2"/>
   <dataValidations count="2">
-    <dataValidation sqref="M2:M5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Aprobado" error="Elegí &quot;sí&quot; o &quot;no&quot;." type="list">
+    <dataValidation sqref="M2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Aprobado" error="Elegí &quot;sí&quot; o &quot;no&quot;." type="list">
       <formula1>"sí,no"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revisó" error="Elegí G (Giuliano) o A (Agustina)." type="list">
+    <dataValidation sqref="N2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revisó" error="Elegí G (Giuliano) o A (Agustina)." type="list">
       <formula1>"G,A"</formula1>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2048,7 +927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P77"/>
+  <dimension ref="A1:P59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4951,48 +3830,48 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a Antigua y Barbuda. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
+          <t>En la base del CIADI hay 0 casos contra Antigua y Barbuda (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a Antigua y Barbuda en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a Antigua y Barbuda entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 0 casos con Antigua y Barbuda como demandado (0 pendientes).
+Búsqueda web ("Eastern Caribbean … expropriation OR nationalisation OR compulsory acquisition foreign company 2020-2026") (https://www.mondaq.com/wealth-management/53510/pirates-of-the-caribbean-expropriation-in-antigua): La expropiación de Half Moon Bay es de 2007, fuera de la ventana.</t>
         </is>
       </c>
       <c r="L41" s="4" t="inlineStr">
@@ -5005,7 +3884,7 @@
       <c r="O41" s="6" t="n"/>
       <c r="P41" s="4" t="inlineStr">
         <is>
-          <t>da36ce560e85</t>
+          <t>0a2e0484933d</t>
         </is>
       </c>
     </row>
@@ -5022,48 +3901,48 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a Bahamas. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
+          <t>En la base del CIADI hay 0 casos contra Bahamas (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a Bahamas en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a Bahamas entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 0 casos con Bahamas como demandado (0 pendientes).
+Búsqueda web ("Eastern Caribbean Antigua Dominica St Lucia St Kitts St Vincent Grenada Barbados Bahamas expropriation OR nationalisation OR compulsory acquisition foreign company 2020-2026") (https://www.mondaq.com/wealth-management/53510/pirates-of-the-caribbean-expropriation-in-antigua): Solo casos anteriores a 2016 (Antigua, Half Moon Bay, 2007).</t>
         </is>
       </c>
       <c r="L42" s="4" t="inlineStr">
@@ -5076,7 +3955,7 @@
       <c r="O42" s="6" t="n"/>
       <c r="P42" s="4" t="inlineStr">
         <is>
-          <t>8fe678b6a0a4</t>
+          <t>bf64099bce10</t>
         </is>
       </c>
     </row>
@@ -5093,48 +3972,48 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a Barbados. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
+          <t>En la base del CIADI hay 0 casos contra Barbados (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
         </is>
       </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a Barbados en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a Barbados entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 0 casos con Barbados como demandado (0 pendientes).
+Búsqueda web ("Eastern Caribbean Antigua Dominica St Lucia St Kitts St Vincent Grenada Barbados Bahamas expropriation OR nationalisation OR compulsory acquisition foreign company 2020-2026") (https://www.mondaq.com/wealth-management/53510/pirates-of-the-caribbean-expropriation-in-antigua): Solo casos anteriores a 2016 (Antigua, Half Moon Bay, 2007).</t>
         </is>
       </c>
       <c r="L43" s="4" t="inlineStr">
@@ -5147,65 +4026,65 @@
       <c r="O43" s="6" t="n"/>
       <c r="P43" s="4" t="inlineStr">
         <is>
-          <t>afcd58bc842c</t>
+          <t>d3ed2729c6a8</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Cuba</t>
+          <t>Costa Rica</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>CUB</t>
+          <t>CRI</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a Cuba. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
+          <t>En la base del CIADI hay 17 casos contra Costa Rica (3 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado).</t>
         </is>
       </c>
       <c r="K44" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a Cuba en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a Cuba entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 17 casos con Costa Rica como demandado (3 pendientes).
+Búsqueda web ("Costa Rica expropiación empresa extranjera 2016-2026") (https://www.ecija.com/actualidad-insights/se-aprueba-nueva-ley-para-atraer-inversionistas-rentistas-y-pensionados-a-costa-rica/): Sin expropiaciones documentadas.</t>
         </is>
       </c>
       <c r="L44" s="4" t="inlineStr">
@@ -5218,65 +4097,65 @@
       <c r="O44" s="6" t="n"/>
       <c r="P44" s="4" t="inlineStr">
         <is>
-          <t>ba1668cc89ea</t>
+          <t>f4b748c69797</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>Dominica</t>
+          <t>Cuba</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>DMA</t>
+          <t>CUB</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a Dominica. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
+          <t>En la base del CIADI hay 0 casos contra Cuba (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
         </is>
       </c>
       <c r="K45" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a Dominica en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a Dominica entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 0 casos con Cuba como demandado (0 pendientes).
+Búsqueda web ("Cuba confiscación nacionalización empresas extranjeras 2022-2025") (https://diariodecuba.com/etiquetas/fihav.html): Sin expropiaciones documentadas; el "corralito" de divisas de 2025 se evaluó en A5.</t>
         </is>
       </c>
       <c r="L45" s="4" t="inlineStr">
@@ -5289,65 +4168,65 @@
       <c r="O45" s="6" t="n"/>
       <c r="P45" s="4" t="inlineStr">
         <is>
-          <t>ec4b0d29cda3</t>
+          <t>cd2418ac25d1</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>El Salvador</t>
+          <t>Dominica</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>SLV</t>
+          <t>DMA</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a El Salvador. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
+          <t>En la base del CIADI hay 0 casos contra Dominica (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
         </is>
       </c>
       <c r="K46" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a El Salvador en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a El Salvador entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 0 casos con Dominica como demandado (0 pendientes).
+Búsqueda web ("Eastern Caribbean Antigua Dominica St Lucia St Kitts St Vincent Grenada Barbados Bahamas expropriation OR nationalisation OR compulsory acquisition foreign company 2020-2026") (https://www.mondaq.com/wealth-management/53510/pirates-of-the-caribbean-expropriation-in-antigua): Solo casos anteriores a 2016 (Antigua, Half Moon Bay, 2007).</t>
         </is>
       </c>
       <c r="L46" s="4" t="inlineStr">
@@ -5360,29 +4239,29 @@
       <c r="O46" s="6" t="n"/>
       <c r="P46" s="4" t="inlineStr">
         <is>
-          <t>c4c3aff7cb79</t>
+          <t>7e7c2e1aa01d</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>El Salvador</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>SLV</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
@@ -5392,33 +4271,33 @@
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 salieron 234 vuelos regulares con pasajeros desde aeropuertos argentinos a Estados Unidos (54,6 por semana en promedio; AMERICAN AIRLINES INC., AEROLINEAS ARGENTINAS SA, LATAM AIRLINES GROUP S.A.(exLAN AIRLINE)).</t>
+          <t>En la base del CIADI hay 6 casos contra El Salvador (1 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>55 vuelos directos por semana en promedio desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado).</t>
         </is>
       </c>
       <c r="K47" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 234 despegues regulares con pasajeros a Estados Unidos en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 14 partidas a Estados Unidos entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 6 casos con El Salvador como demandado (1 pendientes).
+Búsqueda web ("El Salvador expropiación Bukele empresa 2021-2024") (https://diario.elmundo.sv/economia/eeuu-ve-a-el-salvador-atractivo-para-inversion-pero-ve-lentas-las-reformas): Sin expropiaciones documentadas.</t>
         </is>
       </c>
       <c r="L47" s="4" t="inlineStr">
@@ -5431,65 +4310,66 @@
       <c r="O47" s="6" t="n"/>
       <c r="P47" s="4" t="inlineStr">
         <is>
-          <t>80e263c5ded7</t>
+          <t>bd2a9b4b43e4</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>Granada</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>GRD</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a Granada. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
+          <t>En la base del CIADI hay 10 casos contra Estados Unidos (2 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I48" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J48" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado). Caso revisado y no contado: el decomiso del superyate Amadea (2025), por sanciones contra un oligarca ruso. Criterio aprobado (sesión 5): las sanciones internacionales contra personas o entidades puntuales no cuentan como expropiación.</t>
         </is>
       </c>
       <c r="K48" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a Granada en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a Granada entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 10 casos con Estados Unidos como demandado (2 pendientes).
+Radio Free Europe/Radio Liberty, decomiso del superyate Amadea (18/03/2025) (https://www.rferl.org/a/russia-sanctions-yacht-oligarch-amadea/33348093.html): Decomiso judicial de un yate atribuido a un oligarca ruso sancionado. No cuenta (sanción internacional).
+Búsqueda web ("United States government expropriation OR nationalization OR seizure of company assets 2017-2026") (https://corpgov.law.harvard.edu/2015/07/13/illegality-and-hardball-in-governments-nationalization-of-aig/): Solo el caso AIG (2008), fuera de la ventana.</t>
         </is>
       </c>
       <c r="L48" s="4" t="inlineStr">
@@ -5502,65 +4382,65 @@
       <c r="O48" s="6" t="n"/>
       <c r="P48" s="4" t="inlineStr">
         <is>
-          <t>7ffb734e483c</t>
+          <t>66fba037ce8e</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Guatemala</t>
+          <t>Granada</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>GTM</t>
+          <t>GRD</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a Guatemala. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
+          <t>En la base del CIADI hay 5 casos contra Granada (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
         </is>
       </c>
       <c r="K49" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a Guatemala en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a Guatemala entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 5 casos con Granada como demandado (0 pendientes).
+NOW Grenada, arbitraje por las acciones de Grenlec (2017) (https://nowgrenada.com/2017/05/gpp-wrb-file-arbitration-claim-re-grenlec-shares/): Fue una recompra contractual de acciones, resuelta por laudo y acuerdo en 2020; no es una expropiación.</t>
         </is>
       </c>
       <c r="L49" s="4" t="inlineStr">
@@ -5573,65 +4453,65 @@
       <c r="O49" s="6" t="n"/>
       <c r="P49" s="4" t="inlineStr">
         <is>
-          <t>952eec301cfa</t>
+          <t>aa83488694c9</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Haití</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>HTI</t>
+          <t>GTM</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a Haití. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
+          <t>En la base del CIADI hay 8 casos contra Guatemala (2 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado).</t>
         </is>
       </c>
       <c r="K50" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a Haití en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a Haití entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 8 casos con Guatemala como demandado (2 pendientes).
+Búsqueda web ("Guatemala licencia minera suspendida 2022-2024") (https://emisorasunidas.com/2020/06/19/suspension-de-operaciones-de-minera/): Suspensiones de licencias por falta de consulta indígena, no expropiaciones.</t>
         </is>
       </c>
       <c r="L50" s="4" t="inlineStr">
@@ -5644,65 +4524,65 @@
       <c r="O50" s="6" t="n"/>
       <c r="P50" s="4" t="inlineStr">
         <is>
-          <t>da0b897c8cbe</t>
+          <t>c4cc16bd8807</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Honduras</t>
+          <t>Haití</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>HND</t>
+          <t>HTI</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a Honduras. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
+          <t>En la base del CIADI hay 0 casos contra Haití (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
         </is>
       </c>
       <c r="K51" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a Honduras en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a Honduras entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 0 casos con Haití como demandado (0 pendientes).
+Búsqueda web ("Haiti expropriation OR nationalisation foreign company 2021-2026") (https://www.openglobalrights.org/Land-grabs-Haiti-mining-threat-extractives-industry/): Sin expropiaciones documentadas.</t>
         </is>
       </c>
       <c r="L51" s="4" t="inlineStr">
@@ -5715,65 +4595,65 @@
       <c r="O51" s="6" t="n"/>
       <c r="P51" s="4" t="inlineStr">
         <is>
-          <t>48ff9cbd246c</t>
+          <t>c16fd86104ea</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>Honduras</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>JAM</t>
+          <t>HND</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a Jamaica. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
+          <t>En la base del CIADI hay 19 casos contra Honduras (12 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I52" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J52" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado).</t>
         </is>
       </c>
       <c r="K52" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a Jamaica en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a Jamaica entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 19 casos con Honduras como demandado (12 pendientes).
+Búsqueda web ("Honduras expropiación OR nacionalización OR confiscación empresa 2022-2025") (https://www.laprensa.hn/honduras/trabajadores-hondurenos-reclaman-derechos-en-marcha-que-lidero-xiomara-castro-BL7937289): Solo discursos sobre recuperar empresas estatales; ningún caso concreto. Los reclamos ante el CIADI no documentan una expropiación resuelta.</t>
         </is>
       </c>
       <c r="L52" s="4" t="inlineStr">
@@ -5786,65 +4666,65 @@
       <c r="O52" s="6" t="n"/>
       <c r="P52" s="4" t="inlineStr">
         <is>
-          <t>918f55102282</t>
+          <t>5f695242384b</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>Nicaragua</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>NIC</t>
+          <t>JAM</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a Nicaragua. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
+          <t>En la base del CIADI hay 3 casos contra Jamaica (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
         </is>
       </c>
       <c r="K53" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a Nicaragua en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a Nicaragua entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 3 casos con Jamaica como demandado (0 pendientes).
+Búsqueda web ("Trinidad and Tobago OR Jamaica OR Belize … expropriation compulsory acquisition company 2022-2025") (https://bz.vlex.com/vid/british-caribbean-bank-ltd-793042837): En Jamaica y Trinidad y Tobago, sin expropiaciones documentadas en la ventana.</t>
         </is>
       </c>
       <c r="L53" s="4" t="inlineStr">
@@ -5857,7 +4737,7 @@
       <c r="O53" s="6" t="n"/>
       <c r="P53" s="4" t="inlineStr">
         <is>
-          <t>2645784b5ef9</t>
+          <t>69dfd7333f8c</t>
         </is>
       </c>
     </row>
@@ -5874,12 +4754,12 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
@@ -5889,33 +4769,33 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 salieron 357 vuelos regulares con pasajeros desde aeropuertos argentinos a Panamá (83,3 por semana en promedio; COMPAÑIA PANAMEÑA DE AVIACION, SKY HIGH DOMINICANA).</t>
+          <t>En la base del CIADI hay 25 casos contra Panamá (10 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>83 vuelos directos por semana en promedio desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H54" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I54" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J54" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado).</t>
         </is>
       </c>
       <c r="K54" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 357 despegues regulares con pasajeros a Panamá en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 43 partidas a Panamá entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 25 casos con Panamá como demandado (10 pendientes).
+Búsqueda web ("Panamá Corte Suprema Ley 406 First Quantum") (https://www.df.cl/empresas/mineria/corte-suprema-de-panama-revoca-permiso-para-operar-de-first-quantum-y): El cierre de Cobre Panamá fue por la anulación judicial del contrato (evaluada en A5); no hubo expropiación formal. First Quantum reclama ante el CIADI.</t>
         </is>
       </c>
       <c r="L54" s="4" t="inlineStr">
@@ -5928,7 +4808,7 @@
       <c r="O54" s="6" t="n"/>
       <c r="P54" s="4" t="inlineStr">
         <is>
-          <t>964eb808cf11</t>
+          <t>face753d4e1e</t>
         </is>
       </c>
     </row>
@@ -5945,12 +4825,12 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
@@ -5960,33 +4840,33 @@
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 salieron 117 vuelos regulares con pasajeros desde aeropuertos argentinos a República Dominicana (27,3 por semana en promedio; ARAJET (ex DOMINICAN WINGS), AEROLINEAS ARGENTINAS SA).</t>
+          <t>En la base del CIADI hay 4 casos contra República Dominicana (1 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>27 vuelos directos por semana en promedio desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado).</t>
         </is>
       </c>
       <c r="K55" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 117 despegues regulares con pasajeros a República Dominicana en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 25 partidas a República Dominicana entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 4 casos con República Dominicana como demandado (1 pendientes).
+Búsqueda web ("República Dominicana expropiación OR confiscación empresa extranjera 2022-2026") (https://www.elcaribe.com.do/panorama/pais/tc-reitera-que-las-expropiaciones-sin-previo-pago-son-inconstitucionales/): Sin expropiaciones documentadas de empresas en la ventana.</t>
         </is>
       </c>
       <c r="L55" s="4" t="inlineStr">
@@ -5999,7 +4879,7 @@
       <c r="O55" s="6" t="n"/>
       <c r="P55" s="4" t="inlineStr">
         <is>
-          <t>3215383e7153</t>
+          <t>e2b030390583</t>
         </is>
       </c>
     </row>
@@ -6016,48 +4896,48 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a San Cristóbal y Nieves. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
+          <t>En la base del CIADI hay 1 casos contra San Cristóbal y Nieves (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H56" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I56" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J56" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
         </is>
       </c>
       <c r="K56" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a San Cristóbal y Nieves en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a San Cristóbal y Nieves entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 1 casos con San Cristóbal y Nieves como demandado (0 pendientes).
+Búsqueda web ("Eastern Caribbean Antigua Dominica St Lucia St Kitts St Vincent Grenada Barbados Bahamas expropriation OR nationalisation OR compulsory acquisition foreign company 2020-2026") (https://www.mondaq.com/wealth-management/53510/pirates-of-the-caribbean-expropriation-in-antigua): Solo casos anteriores a 2016 (Antigua, Half Moon Bay, 2007).</t>
         </is>
       </c>
       <c r="L56" s="4" t="inlineStr">
@@ -6070,65 +4950,65 @@
       <c r="O56" s="6" t="n"/>
       <c r="P56" s="4" t="inlineStr">
         <is>
-          <t>0dccecba9cc6</t>
+          <t>49d0144e1cca</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>Santa Lucía</t>
+          <t>San Vicente y las Granadinas</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>LCA</t>
+          <t>VCT</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a Santa Lucía. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
+          <t>En la base del CIADI hay 0 casos contra San Vicente y las Granadinas (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
         </is>
       </c>
       <c r="K57" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a Santa Lucía en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a Santa Lucía entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 0 casos con San Vicente y las Granadinas como demandado (0 pendientes).
+Búsqueda web ("Eastern Caribbean Antigua Dominica St Lucia St Kitts St Vincent Grenada Barbados Bahamas expropriation OR nationalisation OR compulsory acquisition foreign company 2020-2026") (https://www.mondaq.com/wealth-management/53510/pirates-of-the-caribbean-expropriation-in-antigua): Solo casos anteriores a 2016 (Antigua, Half Moon Bay, 2007).</t>
         </is>
       </c>
       <c r="L57" s="4" t="inlineStr">
@@ -6141,65 +5021,65 @@
       <c r="O57" s="6" t="n"/>
       <c r="P57" s="4" t="inlineStr">
         <is>
-          <t>82045df1c45b</t>
+          <t>3a016a3140d3</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>Trinidad y Tobago</t>
+          <t>Santa Lucía</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>TTO</t>
+          <t>LCA</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>I3-2</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>¿No hay conexión aérea directa desde Argentina con al menos 3 vuelos semanales?</t>
+          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>En septiembre de 2026 no salieron vuelos regulares con pasajeros desde aeropuertos argentinos a Trinidad y Tobago. Tampoco figuran partidas suficientes en el tablero de Ezeiza y Aeroparque del 26/10 al 01/11/2026 (0).</t>
+          <t>En la base del CIADI hay 1 casos contra Santa Lucía (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>sin vuelos directos regulares desde Argentina (dato 2026, ANAC)</t>
+          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
         </is>
       </c>
       <c r="H58" s="5" t="inlineStr">
         <is>
-          <t>https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv</t>
+          <t>https://icsid.worldbank.org/cases/case-database</t>
         </is>
       </c>
       <c r="I58" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) · 2026-10-28</t>
+          <t>CIADI, base de casos · 2026-10-28</t>
         </is>
       </c>
       <c r="J58" s="4" t="inlineStr">
         <is>
-          <t>Se contaron los despegues internacionales regulares con pasajeros desde todos los aeropuertos argentinos en septiembre de 2026, último mes publicado por la ANAC, y se tomó el promedio semanal (vuelos del mes × 7 / 30). El tablero oficial de Ezeiza y Aeroparque (26/10 al 01/11/2026) se usó como control; esa semana hubo obras en la pista de Ezeiza (25/10 al 11/11/2026) y el tablero no muestra a todas las aerolíneas extranjeras.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
         </is>
       </c>
       <c r="K58" s="4" t="inlineStr">
         <is>
-          <t>ANAC, aterrizajes y despegues procesados (dataset oficial, enero a septiembre de 2026) (https://datos.transporte.gob.ar/dataset/21038a1a-c3c7-4494-b76a-3a2a8fbb83b5/resource/7b6d0103-0a69-4c67-aed9-33cb58ae12f5/download/202609-informe-ministerio-vf-matricula.csv): 0 despegues regulares con pasajeros a Trinidad y Tobago en septiembre de 2026.
-Aeropuertos Argentina, tablero oficial de partidas de Ezeiza y Aeroparque (https://www.aeropuertosargentina.com/vuelos?aeropuerto=EZE&amp;movtp=D): 0 partidas a Trinidad y Tobago entre el 26/10 y el 01/11/2026.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 1 casos con Santa Lucía como demandado (0 pendientes).
+Búsqueda web ("Eastern Caribbean Antigua Dominica St Lucia St Kitts St Vincent Grenada Barbados Bahamas expropriation OR nationalisation OR compulsory acquisition foreign company 2020-2026") (https://www.mondaq.com/wealth-management/53510/pirates-of-the-caribbean-expropriation-in-antigua): Solo casos anteriores a 2016 (Antigua, Half Moon Bay, 2007).</t>
         </is>
       </c>
       <c r="L58" s="4" t="inlineStr">
@@ -6212,19 +5092,19 @@
       <c r="O58" s="6" t="n"/>
       <c r="P58" s="4" t="inlineStr">
         <is>
-          <t>e0a332929aac</t>
+          <t>a3b680a8752d</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>Antigua y Barbuda</t>
+          <t>Trinidad y Tobago</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>ATG</t>
+          <t>TTO</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -6244,7 +5124,7 @@
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>En la base del CIADI hay 0 casos contra Antigua y Barbuda (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
+          <t>En la base del CIADI hay 4 casos contra Trinidad y Tobago (2 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
@@ -6264,13 +5144,13 @@
       </c>
       <c r="J59" s="4" t="inlineStr">
         <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
+          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado).</t>
         </is>
       </c>
       <c r="K59" s="4" t="inlineStr">
         <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 0 casos con Antigua y Barbuda como demandado (0 pendientes).
-Búsqueda web ("Eastern Caribbean … expropriation OR nationalisation OR compulsory acquisition foreign company 2020-2026") (https://www.mondaq.com/wealth-management/53510/pirates-of-the-caribbean-expropriation-in-antigua): La expropiación de Half Moon Bay es de 2007, fuera de la ventana.</t>
+          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 4 casos con Trinidad y Tobago como demandado (2 pendientes).
+Búsqueda web ("Trinidad and Tobago OR Jamaica OR Belize … expropriation compulsory acquisition company 2022-2025") (https://bz.vlex.com/vid/british-caribbean-bank-ltd-793042837): En Jamaica y Trinidad y Tobago, sin expropiaciones documentadas en la ventana.</t>
         </is>
       </c>
       <c r="L59" s="4" t="inlineStr">
@@ -6283,1297 +5163,18 @@
       <c r="O59" s="6" t="n"/>
       <c r="P59" s="4" t="inlineStr">
         <is>
-          <t>0a2e0484933d</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="4" t="inlineStr">
-        <is>
-          <t>Bahamas</t>
-        </is>
-      </c>
-      <c r="B60" s="4" t="inlineStr">
-        <is>
-          <t>BHS</t>
-        </is>
-      </c>
-      <c r="C60" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D60" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E60" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F60" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 0 casos contra Bahamas (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G60" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H60" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I60" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J60" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
-        </is>
-      </c>
-      <c r="K60" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 0 casos con Bahamas como demandado (0 pendientes).
-Búsqueda web ("Eastern Caribbean Antigua Dominica St Lucia St Kitts St Vincent Grenada Barbados Bahamas expropriation OR nationalisation OR compulsory acquisition foreign company 2020-2026") (https://www.mondaq.com/wealth-management/53510/pirates-of-the-caribbean-expropriation-in-antigua): Solo casos anteriores a 2016 (Antigua, Half Moon Bay, 2007).</t>
-        </is>
-      </c>
-      <c r="L60" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M60" s="6" t="n"/>
-      <c r="N60" s="6" t="n"/>
-      <c r="O60" s="6" t="n"/>
-      <c r="P60" s="4" t="inlineStr">
-        <is>
-          <t>bf64099bce10</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="4" t="inlineStr">
-        <is>
-          <t>Barbados</t>
-        </is>
-      </c>
-      <c r="B61" s="4" t="inlineStr">
-        <is>
-          <t>BRB</t>
-        </is>
-      </c>
-      <c r="C61" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D61" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E61" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F61" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 0 casos contra Barbados (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G61" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H61" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I61" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J61" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
-        </is>
-      </c>
-      <c r="K61" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 0 casos con Barbados como demandado (0 pendientes).
-Búsqueda web ("Eastern Caribbean Antigua Dominica St Lucia St Kitts St Vincent Grenada Barbados Bahamas expropriation OR nationalisation OR compulsory acquisition foreign company 2020-2026") (https://www.mondaq.com/wealth-management/53510/pirates-of-the-caribbean-expropriation-in-antigua): Solo casos anteriores a 2016 (Antigua, Half Moon Bay, 2007).</t>
-        </is>
-      </c>
-      <c r="L61" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M61" s="6" t="n"/>
-      <c r="N61" s="6" t="n"/>
-      <c r="O61" s="6" t="n"/>
-      <c r="P61" s="4" t="inlineStr">
-        <is>
-          <t>d3ed2729c6a8</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="4" t="inlineStr">
-        <is>
-          <t>Costa Rica</t>
-        </is>
-      </c>
-      <c r="B62" s="4" t="inlineStr">
-        <is>
-          <t>CRI</t>
-        </is>
-      </c>
-      <c r="C62" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D62" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E62" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F62" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 17 casos contra Costa Rica (3 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G62" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H62" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I62" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J62" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado).</t>
-        </is>
-      </c>
-      <c r="K62" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 17 casos con Costa Rica como demandado (3 pendientes).
-Búsqueda web ("Costa Rica expropiación empresa extranjera 2016-2026") (https://www.ecija.com/actualidad-insights/se-aprueba-nueva-ley-para-atraer-inversionistas-rentistas-y-pensionados-a-costa-rica/): Sin expropiaciones documentadas.</t>
-        </is>
-      </c>
-      <c r="L62" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M62" s="6" t="n"/>
-      <c r="N62" s="6" t="n"/>
-      <c r="O62" s="6" t="n"/>
-      <c r="P62" s="4" t="inlineStr">
-        <is>
-          <t>f4b748c69797</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="4" t="inlineStr">
-        <is>
-          <t>Cuba</t>
-        </is>
-      </c>
-      <c r="B63" s="4" t="inlineStr">
-        <is>
-          <t>CUB</t>
-        </is>
-      </c>
-      <c r="C63" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D63" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E63" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F63" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 0 casos contra Cuba (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G63" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H63" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I63" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J63" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
-        </is>
-      </c>
-      <c r="K63" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 0 casos con Cuba como demandado (0 pendientes).
-Búsqueda web ("Cuba confiscación nacionalización empresas extranjeras 2022-2025") (https://diariodecuba.com/etiquetas/fihav.html): Sin expropiaciones documentadas; el "corralito" de divisas de 2025 se evaluó en A5.</t>
-        </is>
-      </c>
-      <c r="L63" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M63" s="6" t="n"/>
-      <c r="N63" s="6" t="n"/>
-      <c r="O63" s="6" t="n"/>
-      <c r="P63" s="4" t="inlineStr">
-        <is>
-          <t>cd2418ac25d1</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="4" t="inlineStr">
-        <is>
-          <t>Dominica</t>
-        </is>
-      </c>
-      <c r="B64" s="4" t="inlineStr">
-        <is>
-          <t>DMA</t>
-        </is>
-      </c>
-      <c r="C64" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D64" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E64" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F64" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 0 casos contra Dominica (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G64" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H64" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I64" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J64" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
-        </is>
-      </c>
-      <c r="K64" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 0 casos con Dominica como demandado (0 pendientes).
-Búsqueda web ("Eastern Caribbean Antigua Dominica St Lucia St Kitts St Vincent Grenada Barbados Bahamas expropriation OR nationalisation OR compulsory acquisition foreign company 2020-2026") (https://www.mondaq.com/wealth-management/53510/pirates-of-the-caribbean-expropriation-in-antigua): Solo casos anteriores a 2016 (Antigua, Half Moon Bay, 2007).</t>
-        </is>
-      </c>
-      <c r="L64" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M64" s="6" t="n"/>
-      <c r="N64" s="6" t="n"/>
-      <c r="O64" s="6" t="n"/>
-      <c r="P64" s="4" t="inlineStr">
-        <is>
-          <t>7e7c2e1aa01d</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="4" t="inlineStr">
-        <is>
-          <t>El Salvador</t>
-        </is>
-      </c>
-      <c r="B65" s="4" t="inlineStr">
-        <is>
-          <t>SLV</t>
-        </is>
-      </c>
-      <c r="C65" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D65" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E65" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F65" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 6 casos contra El Salvador (1 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G65" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H65" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I65" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J65" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado).</t>
-        </is>
-      </c>
-      <c r="K65" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 6 casos con El Salvador como demandado (1 pendientes).
-Búsqueda web ("El Salvador expropiación Bukele empresa 2021-2024") (https://diario.elmundo.sv/economia/eeuu-ve-a-el-salvador-atractivo-para-inversion-pero-ve-lentas-las-reformas): Sin expropiaciones documentadas.</t>
-        </is>
-      </c>
-      <c r="L65" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M65" s="6" t="n"/>
-      <c r="N65" s="6" t="n"/>
-      <c r="O65" s="6" t="n"/>
-      <c r="P65" s="4" t="inlineStr">
-        <is>
-          <t>bd2a9b4b43e4</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="4" t="inlineStr">
-        <is>
-          <t>Estados Unidos</t>
-        </is>
-      </c>
-      <c r="B66" s="4" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C66" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D66" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E66" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F66" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 10 casos contra Estados Unidos (2 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G66" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H66" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I66" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J66" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado). Caso revisado y no contado: el decomiso del superyate Amadea (2025), por sanciones contra un oligarca ruso. Criterio aprobado (sesión 5): las sanciones internacionales contra personas o entidades puntuales no cuentan como expropiación.</t>
-        </is>
-      </c>
-      <c r="K66" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 10 casos con Estados Unidos como demandado (2 pendientes).
-Radio Free Europe/Radio Liberty, decomiso del superyate Amadea (18/03/2025) (https://www.rferl.org/a/russia-sanctions-yacht-oligarch-amadea/33348093.html): Decomiso judicial de un yate atribuido a un oligarca ruso sancionado. No cuenta (sanción internacional).
-Búsqueda web ("United States government expropriation OR nationalization OR seizure of company assets 2017-2026") (https://corpgov.law.harvard.edu/2015/07/13/illegality-and-hardball-in-governments-nationalization-of-aig/): Solo el caso AIG (2008), fuera de la ventana.</t>
-        </is>
-      </c>
-      <c r="L66" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M66" s="6" t="n"/>
-      <c r="N66" s="6" t="n"/>
-      <c r="O66" s="6" t="n"/>
-      <c r="P66" s="4" t="inlineStr">
-        <is>
-          <t>66fba037ce8e</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="4" t="inlineStr">
-        <is>
-          <t>Granada</t>
-        </is>
-      </c>
-      <c r="B67" s="4" t="inlineStr">
-        <is>
-          <t>GRD</t>
-        </is>
-      </c>
-      <c r="C67" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D67" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 5 casos contra Granada (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G67" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H67" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I67" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J67" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
-        </is>
-      </c>
-      <c r="K67" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 5 casos con Granada como demandado (0 pendientes).
-NOW Grenada, arbitraje por las acciones de Grenlec (2017) (https://nowgrenada.com/2017/05/gpp-wrb-file-arbitration-claim-re-grenlec-shares/): Fue una recompra contractual de acciones, resuelta por laudo y acuerdo en 2020; no es una expropiación.</t>
-        </is>
-      </c>
-      <c r="L67" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M67" s="6" t="n"/>
-      <c r="N67" s="6" t="n"/>
-      <c r="O67" s="6" t="n"/>
-      <c r="P67" s="4" t="inlineStr">
-        <is>
-          <t>aa83488694c9</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="4" t="inlineStr">
-        <is>
-          <t>Guatemala</t>
-        </is>
-      </c>
-      <c r="B68" s="4" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D68" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E68" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F68" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 8 casos contra Guatemala (2 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G68" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H68" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I68" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J68" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado).</t>
-        </is>
-      </c>
-      <c r="K68" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 8 casos con Guatemala como demandado (2 pendientes).
-Búsqueda web ("Guatemala licencia minera suspendida 2022-2024") (https://emisorasunidas.com/2020/06/19/suspension-de-operaciones-de-minera/): Suspensiones de licencias por falta de consulta indígena, no expropiaciones.</t>
-        </is>
-      </c>
-      <c r="L68" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M68" s="6" t="n"/>
-      <c r="N68" s="6" t="n"/>
-      <c r="O68" s="6" t="n"/>
-      <c r="P68" s="4" t="inlineStr">
-        <is>
-          <t>c4cc16bd8807</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="4" t="inlineStr">
-        <is>
-          <t>Haití</t>
-        </is>
-      </c>
-      <c r="B69" s="4" t="inlineStr">
-        <is>
-          <t>HTI</t>
-        </is>
-      </c>
-      <c r="C69" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D69" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 0 casos contra Haití (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G69" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H69" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I69" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J69" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
-        </is>
-      </c>
-      <c r="K69" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 0 casos con Haití como demandado (0 pendientes).
-Búsqueda web ("Haiti expropriation OR nationalisation foreign company 2021-2026") (https://www.openglobalrights.org/Land-grabs-Haiti-mining-threat-extractives-industry/): Sin expropiaciones documentadas.</t>
-        </is>
-      </c>
-      <c r="L69" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M69" s="6" t="n"/>
-      <c r="N69" s="6" t="n"/>
-      <c r="O69" s="6" t="n"/>
-      <c r="P69" s="4" t="inlineStr">
-        <is>
-          <t>c16fd86104ea</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="4" t="inlineStr">
-        <is>
-          <t>Honduras</t>
-        </is>
-      </c>
-      <c r="B70" s="4" t="inlineStr">
-        <is>
-          <t>HND</t>
-        </is>
-      </c>
-      <c r="C70" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D70" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E70" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F70" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 19 casos contra Honduras (12 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G70" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H70" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I70" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J70" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado).</t>
-        </is>
-      </c>
-      <c r="K70" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 19 casos con Honduras como demandado (12 pendientes).
-Búsqueda web ("Honduras expropiación OR nacionalización OR confiscación empresa 2022-2025") (https://www.laprensa.hn/honduras/trabajadores-hondurenos-reclaman-derechos-en-marcha-que-lidero-xiomara-castro-BL7937289): Solo discursos sobre recuperar empresas estatales; ningún caso concreto. Los reclamos ante el CIADI no documentan una expropiación resuelta.</t>
-        </is>
-      </c>
-      <c r="L70" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M70" s="6" t="n"/>
-      <c r="N70" s="6" t="n"/>
-      <c r="O70" s="6" t="n"/>
-      <c r="P70" s="4" t="inlineStr">
-        <is>
-          <t>5f695242384b</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="4" t="inlineStr">
-        <is>
-          <t>Jamaica</t>
-        </is>
-      </c>
-      <c r="B71" s="4" t="inlineStr">
-        <is>
-          <t>JAM</t>
-        </is>
-      </c>
-      <c r="C71" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D71" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E71" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F71" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 3 casos contra Jamaica (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G71" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H71" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I71" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J71" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
-        </is>
-      </c>
-      <c r="K71" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 3 casos con Jamaica como demandado (0 pendientes).
-Búsqueda web ("Trinidad and Tobago OR Jamaica OR Belize … expropriation compulsory acquisition company 2022-2025") (https://bz.vlex.com/vid/british-caribbean-bank-ltd-793042837): En Jamaica y Trinidad y Tobago, sin expropiaciones documentadas en la ventana.</t>
-        </is>
-      </c>
-      <c r="L71" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M71" s="6" t="n"/>
-      <c r="N71" s="6" t="n"/>
-      <c r="O71" s="6" t="n"/>
-      <c r="P71" s="4" t="inlineStr">
-        <is>
-          <t>69dfd7333f8c</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="4" t="inlineStr">
-        <is>
-          <t>Panamá</t>
-        </is>
-      </c>
-      <c r="B72" s="4" t="inlineStr">
-        <is>
-          <t>PAN</t>
-        </is>
-      </c>
-      <c r="C72" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D72" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E72" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F72" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 25 casos contra Panamá (10 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G72" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H72" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I72" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J72" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado).</t>
-        </is>
-      </c>
-      <c r="K72" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 25 casos con Panamá como demandado (10 pendientes).
-Búsqueda web ("Panamá Corte Suprema Ley 406 First Quantum") (https://www.df.cl/empresas/mineria/corte-suprema-de-panama-revoca-permiso-para-operar-de-first-quantum-y): El cierre de Cobre Panamá fue por la anulación judicial del contrato (evaluada en A5); no hubo expropiación formal. First Quantum reclama ante el CIADI.</t>
-        </is>
-      </c>
-      <c r="L72" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M72" s="6" t="n"/>
-      <c r="N72" s="6" t="n"/>
-      <c r="O72" s="6" t="n"/>
-      <c r="P72" s="4" t="inlineStr">
-        <is>
-          <t>face753d4e1e</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="4" t="inlineStr">
-        <is>
-          <t>República Dominicana</t>
-        </is>
-      </c>
-      <c r="B73" s="4" t="inlineStr">
-        <is>
-          <t>DOM</t>
-        </is>
-      </c>
-      <c r="C73" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D73" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E73" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F73" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 4 casos contra República Dominicana (1 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G73" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H73" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I73" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J73" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado).</t>
-        </is>
-      </c>
-      <c r="K73" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 4 casos con República Dominicana como demandado (1 pendientes).
-Búsqueda web ("República Dominicana expropiación OR confiscación empresa extranjera 2022-2026") (https://www.elcaribe.com.do/panorama/pais/tc-reitera-que-las-expropiaciones-sin-previo-pago-son-inconstitucionales/): Sin expropiaciones documentadas de empresas en la ventana.</t>
-        </is>
-      </c>
-      <c r="L73" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M73" s="6" t="n"/>
-      <c r="N73" s="6" t="n"/>
-      <c r="O73" s="6" t="n"/>
-      <c r="P73" s="4" t="inlineStr">
-        <is>
-          <t>e2b030390583</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="4" t="inlineStr">
-        <is>
-          <t>San Cristóbal y Nieves</t>
-        </is>
-      </c>
-      <c r="B74" s="4" t="inlineStr">
-        <is>
-          <t>KNA</t>
-        </is>
-      </c>
-      <c r="C74" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D74" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E74" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F74" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 1 casos contra San Cristóbal y Nieves (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G74" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H74" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I74" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J74" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
-        </is>
-      </c>
-      <c r="K74" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 1 casos con San Cristóbal y Nieves como demandado (0 pendientes).
-Búsqueda web ("Eastern Caribbean Antigua Dominica St Lucia St Kitts St Vincent Grenada Barbados Bahamas expropriation OR nationalisation OR compulsory acquisition foreign company 2020-2026") (https://www.mondaq.com/wealth-management/53510/pirates-of-the-caribbean-expropriation-in-antigua): Solo casos anteriores a 2016 (Antigua, Half Moon Bay, 2007).</t>
-        </is>
-      </c>
-      <c r="L74" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M74" s="6" t="n"/>
-      <c r="N74" s="6" t="n"/>
-      <c r="O74" s="6" t="n"/>
-      <c r="P74" s="4" t="inlineStr">
-        <is>
-          <t>49d0144e1cca</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="4" t="inlineStr">
-        <is>
-          <t>San Vicente y las Granadinas</t>
-        </is>
-      </c>
-      <c r="B75" s="4" t="inlineStr">
-        <is>
-          <t>VCT</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D75" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 0 casos contra San Vicente y las Granadinas (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G75" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H75" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I75" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J75" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
-        </is>
-      </c>
-      <c r="K75" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 0 casos con San Vicente y las Granadinas como demandado (0 pendientes).
-Búsqueda web ("Eastern Caribbean Antigua Dominica St Lucia St Kitts St Vincent Grenada Barbados Bahamas expropriation OR nationalisation OR compulsory acquisition foreign company 2020-2026") (https://www.mondaq.com/wealth-management/53510/pirates-of-the-caribbean-expropriation-in-antigua): Solo casos anteriores a 2016 (Antigua, Half Moon Bay, 2007).</t>
-        </is>
-      </c>
-      <c r="L75" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M75" s="6" t="n"/>
-      <c r="N75" s="6" t="n"/>
-      <c r="O75" s="6" t="n"/>
-      <c r="P75" s="4" t="inlineStr">
-        <is>
-          <t>3a016a3140d3</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="4" t="inlineStr">
-        <is>
-          <t>Santa Lucía</t>
-        </is>
-      </c>
-      <c r="B76" s="4" t="inlineStr">
-        <is>
-          <t>LCA</t>
-        </is>
-      </c>
-      <c r="C76" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D76" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F76" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 1 casos contra Santa Lucía (0 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G76" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H76" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I76" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J76" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO.</t>
-        </is>
-      </c>
-      <c r="K76" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 1 casos con Santa Lucía como demandado (0 pendientes).
-Búsqueda web ("Eastern Caribbean Antigua Dominica St Lucia St Kitts St Vincent Grenada Barbados Bahamas expropriation OR nationalisation OR compulsory acquisition foreign company 2020-2026") (https://www.mondaq.com/wealth-management/53510/pirates-of-the-caribbean-expropriation-in-antigua): Solo casos anteriores a 2016 (Antigua, Half Moon Bay, 2007).</t>
-        </is>
-      </c>
-      <c r="L76" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M76" s="6" t="n"/>
-      <c r="N76" s="6" t="n"/>
-      <c r="O76" s="6" t="n"/>
-      <c r="P76" s="4" t="inlineStr">
-        <is>
-          <t>a3b680a8752d</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="4" t="inlineStr">
-        <is>
-          <t>Trinidad y Tobago</t>
-        </is>
-      </c>
-      <c r="B77" s="4" t="inlineStr">
-        <is>
-          <t>TTO</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>I3-2</t>
-        </is>
-      </c>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo expropiación, nacionalización o confiscación de activos, en cualquier sector, en los últimos 10 años?</t>
-        </is>
-      </c>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
-        <is>
-          <t>En la base del CIADI hay 4 casos contra Trinidad y Tobago (2 pendientes). Ninguna fuente revisada documenta una expropiación, nacionalización o confiscación en los últimos 10 años que cumpla el criterio.</t>
-        </is>
-      </c>
-      <c r="G77" s="4" t="inlineStr">
-        <is>
-          <t>búsqueda en la base del CIADI y en prensa (dato 2026, CIADI y prensa)</t>
-        </is>
-      </c>
-      <c r="H77" s="5" t="inlineStr">
-        <is>
-          <t>https://icsid.worldbank.org/cases/case-database</t>
-        </is>
-      </c>
-      <c r="I77" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J77" s="4" t="inlineStr">
-        <is>
-          <t>Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Una demanda sin resolver no alcanza (criterio aprobado).</t>
-        </is>
-      </c>
-      <c r="K77" s="4" t="inlineStr">
-        <is>
-          <t>CIADI, base de casos (https://icsid.worldbank.org/cases/case-database): 4 casos con Trinidad y Tobago como demandado (2 pendientes).
-Búsqueda web ("Trinidad and Tobago OR Jamaica OR Belize … expropriation compulsory acquisition company 2022-2025") (https://bz.vlex.com/vid/british-caribbean-bank-ltd-793042837): En Jamaica y Trinidad y Tobago, sin expropiaciones documentadas en la ventana.</t>
-        </is>
-      </c>
-      <c r="L77" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M77" s="6" t="n"/>
-      <c r="N77" s="6" t="n"/>
-      <c r="O77" s="6" t="n"/>
-      <c r="P77" s="4" t="inlineStr">
-        <is>
           <t>6aaec61172eb</t>
         </is>
       </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
-  <autoFilter ref="A1:O77"/>
+  <autoFilter ref="A1:O59"/>
   <dataValidations count="2">
-    <dataValidation sqref="M2:M77" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Aprobado" error="Elegí &quot;sí&quot; o &quot;no&quot;." type="list">
+    <dataValidation sqref="M2:M59" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Aprobado" error="Elegí &quot;sí&quot; o &quot;no&quot;." type="list">
       <formula1>"sí,no"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N77" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revisó" error="Elegí G (Giuliano) o A (Agustina)." type="list">
+    <dataValidation sqref="N2:N59" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revisó" error="Elegí G (Giuliano) o A (Agustina)." type="list">
       <formula1>"G,A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7636,24 +5237,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId76"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sesión 6: decisiones de los fundadores (criterios 23 a 25), alertas y A3 con el acuerdo concreto
- Criterio 23 precisado: solo una derogación o anulación definitiva revierte (NO + alerta);
  Estados Unidos A5 sigue en SÍ con alerta del estado judicial de Revolution Wind.
- Criterio 24: C2 con dimensiones disponibles solo si hay al menos 4 de 6.
- Criterio 25: alerta fija por sanciones amplias de EE.UU. (OFAC); aplicada a Cuba.
- Alertas con fuente propia y alertas_pais en calcular.js.
- A3 de los socios de la ALADI cita el ACE vigente y vuelve a revisión.
- Bélgica y Luxemburgo A1 pendientes de consulta a la Dirección de Tratados.
- Confirmaciones de Giuliano registradas. Planillas de pendientes regeneradas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzD7QUUB49X53DnDPTty9t
</commit_message>
<xml_diff>
--- a/data/revision/revision_tanda2_america.xlsx
+++ b/data/revision/revision_tanda2_america.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -551,7 +551,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>- Revisión completa (1 filas): Revisar todas: respuestas interpretativas, en null, fuera del cálculo y todas las condiciones críticas (⚡).</t>
+          <t>- Revisión completa (0 filas): Revisar todas: respuestas interpretativas, en null, fuera del cálculo y todas las condiciones críticas (⚡).</t>
         </is>
       </c>
     </row>
@@ -581,13 +581,6 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>- Canadá A5: Corrección pedida en la revisión de G (planilla revision_tanda2_america, 28/10/2026): como la ley retroactiva se derogó y se devolvió lo cobrado, no cuenta como cambio retroactivo vigente (NO) y se publica como alerta. Reemplaza, para estos casos, el criterio 17 de la sesión 5. A CONFIRMAR.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>- Estados Unidos C3: Búsqueda documentada: no se encontraron casos que cumplan el criterio, así que la respuesta es NO. Caso revisado y no contado: en noviembre de 2022 EE.UU. impuso derechos antidumping a los tubos OCTG argentinos que exporta Siderca (grupo Techint), y Argentina llevó el caso a la OMC (DS617). Criterio aprobado (sesión 5): las medidas antidumping no cuentan como discriminación, salvo que un fallo de la OMC las declare incompatibles. El panel entregó su informe a las partes el 02/05/2025, pero a pedido de ambas su publicación se postergó hasta el 29/10/2026: todavía no hay fallo público. REVISAR DESPUÉS DEL 29/10/2026: si el informe declara la medida incompatible, la respuesta pasa a SÍ.</t>
         </is>
@@ -605,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -708,77 +701,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Canadá</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>CAN</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>A5</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>¿Hubo cambios regulatorios retroactivos documentados en los últimos 5 años, en cualquier sector, que afectaran a empresas extranjeras?</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>La Ley del Impuesto sobre los Servicios Digitales (sanción del 20/06/2024) creó un impuesto de 3% sobre ingresos digitales de grandes empresas, en su mayoría extranjeras, con efecto retroactivo al 01/01/2022. La Ley de Implementación del Presupuesto 2025 n.º 1 (S.C. 2026, c. 3, art. 126), sancionada el 26/03/2026, lo derogó con efecto al 20/06/2024 y ordenó devolver lo cobrado.</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>impuesto retroactivo a los servicios digitales derogado en 2026, con devolución de lo cobrado (dato 2026, BLG)</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>https://www.blg.com/en/insights/2024/07/canadas-unilateral-digital-services-tax-forges-ahead-with-retroactive-effect</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>BLG (Borden Ladner Gervais), "Canada’s unilateral Digital Services Tax forges ahead with retroactive effect" (10/07/2024) · 2026-10-28</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>Corrección pedida en la revisión de G (planilla revision_tanda2_america, 28/10/2026): como la ley retroactiva se derogó y se devolvió lo cobrado, no cuenta como cambio retroactivo vigente (NO) y se publica como alerta. Reemplaza, para estos casos, el criterio 17 de la sesión 5. A CONFIRMAR.</t>
-        </is>
-      </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>Gobierno de Canadá, Justice Laws, Budget 2025 Implementation Act, No. 1 (S.C. 2026, c. 3), art. 126 (https://laws-lois.justice.gc.ca/eng/acts/B-9.8598/FullText.html): Deroga la Ley del Impuesto sobre los Servicios Digitales con efecto al 20/06/2024; sancionada el 26/03/2026.
-PwC Canadá, "Canada intends to rescind its Digital Services Tax Act" (2025) (https://www.pwc.com/ca/en/services/tax/publications/tax-insights/canada-digital-services-tax-act-2025.html): Confirma el efecto retroactivo y el anuncio de derogación de junio de 2025.</t>
-        </is>
-      </c>
-      <c r="L2" s="4" t="inlineStr">
-        <is>
-          <t>pendiente_revision</t>
-        </is>
-      </c>
-      <c r="M2" s="6" t="n"/>
-      <c r="N2" s="6" t="n"/>
-      <c r="O2" s="6" t="n"/>
-      <c r="P2" s="4" t="inlineStr">
-        <is>
-          <t>244cc2c1ef00</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <autoFilter ref="A1:O2"/>
@@ -790,9 +712,6 @@
       <formula1>"G,A"</formula1>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>